<commit_message>
Add dropdown test automation with Excel data
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData1.xlsx
+++ b/src/test/resources/TestData1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="10905" windowHeight="6615"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="11100" windowHeight="2985" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -12,12 +12,12 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="A1:K8"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>FirstNmae</t>
   </si>
@@ -41,6 +41,24 @@
   </si>
   <si>
     <t>Sample test</t>
+  </si>
+  <si>
+    <t>Language</t>
+  </si>
+  <si>
+    <t>IDE</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>Maven</t>
+  </si>
+  <si>
+    <t>CSS</t>
   </si>
 </sst>
 </file>
@@ -435,9 +453,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>